<commit_message>
Responsive + ajout crédits + Maj PopUp
</commit_message>
<xml_diff>
--- a/liste_eleves.xlsx
+++ b/liste_eleves.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t xml:space="preserve">Prénom NOM DE FAMILLE</t>
   </si>
@@ -29,9 +29,6 @@
   </si>
   <si>
     <t xml:space="preserve">Ornella ANTONY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-2026</t>
   </si>
   <si>
     <t xml:space="preserve">Niel ARMENGAUD</t>
@@ -159,11 +156,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -294,6 +291,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -308,140 +306,137 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="0" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>3</v>
+      <c r="B3" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>3</v>
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>3</v>
+        <v>9</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>3</v>
+        <v>10</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>3</v>
+      <c r="B12" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="1"/>
+      <c r="A16" s="0"/>
+      <c r="B16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="2"/>
+      <c r="A17" s="0"/>
+      <c r="B17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="2"/>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="1"/>
+      <c r="A18" s="0"/>
+      <c r="B18" s="0"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2"/>
+      <c r="B20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="1"/>
+      <c r="B21" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="2"/>
+      <c r="B23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="2"/>
+      <c r="B24" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>